<commit_message>
Fix false 'None found' from page scans; guard same-day snapshot overwrite
An 'html' page scan can only prove presence. Previously a scan that found no
AE keywords fell through to 'None found', asserting an empty board when the
real cause was usually a JS shell whose listings never rendered (Granicus,
Polimorphic, Tyler all reported 'None found' off pure nav chrome). A false
'None found' silently hides a warm door, so it now reports Unknown unless the
page explicitly says it has no openings.

Also: refresh.py refused nothing when a snapshot already existed for today,
so a same-day re-run destroyed the prior baseline and left the diff with no
comparison point. It now requires --force and diffs against that run.
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Safety" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Works" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General Gov" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parks &amp; Rec" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K-12 Schools" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transit &amp; Parking" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Public Safety" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Public Works" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="General Gov" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Parks &amp; Rec" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="K-12 Schools" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transit &amp; Parking" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Public Safety'!$A$1:$F$36</definedName>
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -174,8 +174,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -183,10 +183,9 @@
     <xf numFmtId="1" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -204,8 +203,8 @@
     <xf numFmtId="1" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -213,9 +212,9 @@
     <xf numFmtId="1" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -750,7 +749,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>None found - site: 8 roles, none sales</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -780,7 +779,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>None found - eng roles only</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -810,7 +809,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Yes - Strat Accts Sales Mgr</t>
+          <t>Yes - Senior Enterprise Account Executiv (San Francisco, Cal)</t>
         </is>
       </c>
     </row>
@@ -840,7 +839,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Unknown - careers page blocked</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -868,9 +867,9 @@
           <t>Cloud fire department suite: pre-incident planning, RMS, scheduling, and response</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - SDR opening only</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -900,7 +899,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Unknown - careers JS-walled</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -930,7 +929,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>None found - open application only</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -960,7 +959,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>None found - no roles on site</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -990,7 +989,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>None found - site: eng roles only</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1019,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>None found - site board empty</t>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -1048,9 +1047,9 @@
           <t>Body cameras, TASER energy weapons, digital evidence cloud, and real-time operations</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Yes - Sr Enterprise AE +</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -1078,9 +1077,9 @@
           <t>Radios, 911 call handling, CAD, and video security (Avigilon) for public safety</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE reqs on Workday</t>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive Germany (Germany Offsite (Z)</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1109,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Yes - Local &amp; Strategic AE</t>
+          <t>Yes - Regional Account Executive (TN/KY) (Chicago, IL)</t>
         </is>
       </c>
     </row>
@@ -1138,9 +1137,9 @@
           <t>Autonomous drones for police DFR programs and public-sector inspection</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE West Coast</t>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1169,7 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Yes - AE Fire; ASM East</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -1198,9 +1197,9 @@
           <t>Cloud-native CAD and records management (RMS) for law enforcement</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Regional AE - Florida</t>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Software (Manchester)</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1229,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Yes - Federal + CA Growth AE</t>
+          <t>Yes - Federal Account Executive (Washington, D.C.)</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1259,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>None found - ATS: no openings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -1288,9 +1287,9 @@
           <t>Solar-powered mobile surveillance units for cities, retail, and infrastructure</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Strat Rev Exec</t>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1318,9 +1317,9 @@
           <t>AI analysis of body-camera audio for officer professionalism and supervision</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sr AE SW $200-400k OTE</t>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive, Southwes (United States)</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1349,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>None found - no open roles</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -1378,9 +1377,9 @@
           <t>ePCR, records, and analytics connecting EMS, fire, and hospitals</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Regional AE EMS/Fire</t>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Regional Account Executive EMS/Fir (Remote, Pennsylvan)</t>
         </is>
       </c>
     </row>
@@ -1408,9 +1407,9 @@
           <t>Incident records and ePCR data platform for EMS and fire agencies</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - VP Sales + Fed Dir</t>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -1438,9 +1437,9 @@
           <t>Intelligent 911 platform streaming device location and data to dispatch</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>None found - no sales reqs</t>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Join our Go-To-Market Talent Commu only</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1469,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>None found - no open roles</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1498,9 +1497,9 @@
           <t>Assistive AI for 911 centers: transcription, translation, text-to-911, and video</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Strategic AE + SDR</t>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1529,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>Yes - Territory Mgrs + RSMs</t>
+          <t>Yes - Account Executive - TherOx (SS02)  (6 Locations)</t>
         </is>
       </c>
     </row>
@@ -1558,9 +1557,9 @@
           <t>Real-time EMS-to-hospital communication and patient handoff platform</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>None found - general app only</t>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1589,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1619,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>None found - all eng/ops</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1649,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>None found - physician role only</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -1678,9 +1677,9 @@
           <t>Mass notification and critical event management platform</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE roles UK/Germany</t>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (United Kingdom)</t>
         </is>
       </c>
     </row>
@@ -1708,9 +1707,9 @@
           <t>Panic button, 911 data, and community alerting suite (Motorola)</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>Yes - Motorola CCS AE remote</t>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1739,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>None found - eng/support only</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1769,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>None found - accountant only</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1861,7 @@
       </c>
       <c r="F2" s="14" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Key Account Mgr</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1890,9 +1889,9 @@
           <t>Routing, in-cab fleet tech, and resident apps for waste operations</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE Munis, Mtn West</t>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1921,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>Yes - AE Boston/London</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1951,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>None found - no open roles</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -1980,9 +1979,9 @@
           <t>AI recycling-sorting robots and real-time bale/line data</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>None found - AE West removed Jan 26</t>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -2010,9 +2009,9 @@
           <t>AI waste-recognition cameras and analytics for sorting plants</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - VP Sales London</t>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2041,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>None found - tech roles only</t>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2071,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2101,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Yes - Territory Mgr PacNW</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2131,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>None found - cust care only</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2161,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Yes - AEs VA/MD/NY/WA/UT</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2191,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Yes - Strategic AE (NY!)</t>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -2220,9 +2219,9 @@
           <t>AI roadway intelligence: ALPR, traffic monitoring, incident detection</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>Unknown - ADP portal JS-walled</t>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -2250,9 +2249,9 @@
           <t>Traffic data collection and smart intersection technology</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Ent AE Opticom SE US</t>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Account Executive, Opti (Southeastern USA)</t>
         </is>
       </c>
     </row>
@@ -2280,9 +2279,9 @@
           <t>AI-powered traffic signal optimization platform</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>None found - site board: 0 jobs</t>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2311,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>None found - 19 roles, all technical</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2341,7 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>Yes - AE San Carlos (site)</t>
+          <t>Yes - Account Executive ( College Park, MD)</t>
         </is>
       </c>
     </row>
@@ -2370,9 +2369,9 @@
           <t>School bus stop-arm cameras with violator-funded safety programs</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - VP Reg Sales NE open</t>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Regional Account Executive, DE, MD (US - Remote)</t>
         </is>
       </c>
     </row>
@@ -2400,9 +2399,9 @@
           <t>Speed, volume, and congestion analytics for public works and police</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>Yes - AE, Jacksonville</t>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.urbansdk.com/ca</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2431,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -2460,9 +2459,9 @@
           <t>Tolling and intelligent transportation systems (owns IRD, ETC); acquiring Conduent's tolling unit</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>None found - no sales listings</t>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2490,9 +2489,9 @@
           <t>Government services giant (Xerox spinoff): transit fare, payments, DMV; selling tolling to Quarterhill</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Exec Tolling</t>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2521,7 @@
       </c>
       <c r="F24" s="15" t="inlineStr">
         <is>
-          <t>Yes - Sr AE Boston (site)</t>
+          <t>Yes - Senior Account Executive (Boston, Massachuse)</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2551,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>None found - no jobs on YC page</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2582,7 +2581,7 @@
       </c>
       <c r="F26" s="15" t="inlineStr">
         <is>
-          <t>Yes - RSM + field sales open</t>
+          <t>Yes - Key Account Manager (Budapest, Hungary)</t>
         </is>
       </c>
     </row>
@@ -2610,9 +2609,9 @@
           <t>Water meters and ORION AMI networks for utilities</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Municipal AM MD/SoCal</t>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager- Private Water (4 Locations)</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2641,7 @@
       </c>
       <c r="F28" s="15" t="inlineStr">
         <is>
-          <t>Yes - Territory Mgrs NC/OH/CO</t>
+          <t>Yes - Jr. Sales Representative (Remote - Tennessee)</t>
         </is>
       </c>
     </row>
@@ -2670,9 +2669,9 @@
           <t>Lead service line inventories, sampling, and compliance software</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>None found - AE closed 6+ mo ago</t>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2701,7 @@
       </c>
       <c r="F30" s="15" t="inlineStr">
         <is>
-          <t>Yes - Strategic AE TX/remote</t>
+          <t>Yes - Strategic Account Executive - Texa</t>
         </is>
       </c>
     </row>
@@ -2730,9 +2729,9 @@
           <t>AI pipe-failure prediction for main replacement planning</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE Central US</t>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2760,9 +2759,9 @@
           <t>Automated water quality monitoring as a service</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2791,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>None found - sales posts expired</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -2820,9 +2819,9 @@
           <t>AI defect detection and coding for sewer inspection video</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
-        <is>
-          <t>None found - AE posting 404s</t>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive, Enterprise (Remote)</t>
         </is>
       </c>
     </row>
@@ -2850,9 +2849,9 @@
           <t>Robotic sewer inspection and condition assessment services</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Regional Sales Mgr</t>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2880,9 +2879,9 @@
           <t>ArcGIS - the mapping and asset data backbone of most public works departments</t>
         </is>
       </c>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>Yes - GIS Account Manager</t>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -2910,9 +2909,9 @@
           <t>IoT telematics and video safety for government fleets (public co)</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Major AE, remote</t>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2941,7 @@
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Yes - Technical AE, remote</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -2970,9 +2969,9 @@
           <t>Asset and work order management for DPWs (part of OpenGov)</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>Yes - OpenGov AE Chicago</t>
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -3000,9 +2999,9 @@
           <t>Asset management ex-Dude Solutions, now Siemens-owned</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
-        <is>
-          <t>Yes - Sr Acct Mgr Education NC</t>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -3037,64 +3036,64 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Vantiq</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Walnut Creek, CA</t>
         </is>
       </c>
-      <c r="C2" s="20" t="n">
+      <c r="C2" s="19" t="n">
         <v>2015</v>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Citizen Services</t>
         </is>
       </c>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Real-time agentic AI platform used for smart city and public service monitoring</t>
         </is>
       </c>
-      <c r="F2" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - careers JS-walled</t>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -3122,39 +3121,39 @@
           <t>Resident communications (govDelivery), meeting and agenda management, digital services</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE Midwest remote</t>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>CivicPlus</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Manhattan, KS</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="19" t="n">
         <v>1994</v>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Citizen Services</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Municipal websites, 311/CRM, mass notification, and agenda software</t>
         </is>
       </c>
-      <c r="F4" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE, remote</t>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -3182,39 +3181,39 @@
           <t>AI voice and chat agents plus constituent CRM for local governments</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior AE, remote</t>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Polco</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Madison, WI</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="19" t="n">
         <v>2015</v>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Citizen Services</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Community surveys, benchmarking, and budget simulation (owns National Research Center)</t>
         </is>
       </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE remote $80-115k</t>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -3242,39 +3241,39 @@
           <t>Permitting, licensing, and code enforcement platform for state and local government</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE remote US</t>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Remote Based - US)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>OpenGov</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>San Jose, CA</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="19" t="n">
         <v>2012</v>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Permitting &amp; Licensing</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Permitting, budgeting, procurement, and asset management cloud suite (Cox-owned)</t>
         </is>
       </c>
-      <c r="F8" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE + 3 Ent AE Chi/Bos</t>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -3304,37 +3303,37 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>None found - 8 roles, no sales</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>GovWell</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="19" t="n">
         <v>2023</v>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Permitting &amp; Licensing</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>AI permitting and licensing platform: 24/7 resident assistant, AI code-compliance review</t>
         </is>
       </c>
-      <c r="F10" s="22" t="inlineStr">
-        <is>
-          <t>Yes - SMB Gov AE, NYC</t>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Small &amp; Medium (New York, NY)</t>
         </is>
       </c>
     </row>
@@ -3362,39 +3361,39 @@
           <t>AI cameras on city fleet vehicles detect blight, graffiti, dumping for code enforcement</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE remote $85-95k</t>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Tyler Technologies</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Plano, TX</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="19" t="n">
         <v>1966</v>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Finance &amp; ERP</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>The govtech giant: ERP, courts, public safety, permitting, and payments</t>
         </is>
       </c>
-      <c r="F12" s="22" t="inlineStr">
-        <is>
-          <t>Yes - many AEs; ERP AE West</t>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -3424,37 +3423,37 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Unknown - careers JS-walled</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>ClearGov</t>
         </is>
       </c>
-      <c r="B14" s="19" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Maynard, MA</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="19" t="n">
         <v>2015</v>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Finance &amp; ERP</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>Budget building and transparency software for local governments and schools</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>Yes - AE, remote</t>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -3482,39 +3481,39 @@
           <t>Treasury platform for local government finance teams: AI reconciliation and cash forecasting</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - BDR only</t>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Pavilion</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="19" t="n">
         <v>2018</v>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>Procurement &amp; Payments</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>Free search marketplace for cooperative contracts (formerly CoProcure)</t>
         </is>
       </c>
-      <c r="F16" s="23" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - BD Associate only</t>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 405 for https://www.withpavilion.co</t>
         </is>
       </c>
     </row>
@@ -3542,39 +3541,39 @@
           <t>Government purchasing data and procurement intelligence (ex-SmartProcure)</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE remote FL/VA</t>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>PayIt</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Kansas City, MO</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="19" t="n">
         <v>2013</v>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Procurement &amp; Payments</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>Digital services and payments platform for state and local government</t>
         </is>
       </c>
-      <c r="F18" s="21" t="inlineStr">
-        <is>
-          <t>None found - site board: no sales</t>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -3604,37 +3603,37 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Unknown - own ATS not readable</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>InvoiceCloud</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>Braintree, MA</t>
         </is>
       </c>
-      <c r="C20" s="20" t="n">
+      <c r="C20" s="19" t="n">
         <v>2009</v>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Procurement &amp; Payments</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>Electronic billing and payments for local government and utilities</t>
         </is>
       </c>
-      <c r="F20" s="22" t="inlineStr">
-        <is>
-          <t>Yes - MM AE Boston + Acct Dirs</t>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Yes - Mid Market Account Executive (Boston, MA)</t>
         </is>
       </c>
     </row>
@@ -3662,39 +3661,39 @@
           <t>Public-sector HR suite: recruiting, onboarding, and performance</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - site blocked; AE indexed</t>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>UKG</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>Lowell, MA</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="19" t="n">
         <v>2020</v>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>HR &amp; Workforce</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>Workforce management giant (Kronos + Ultimate merger) with large gov base</t>
         </is>
       </c>
       <c r="F22" s="22" t="inlineStr">
         <is>
-          <t>Yes - multiple AEs, own site</t>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -3722,39 +3721,39 @@
           <t>Pension, OPEB, and labor cost analytics for governments</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Yes - TrueComp MM AE remote</t>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Mid-Market Account Executive</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Holly</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="19" t="n">
         <v>2023</v>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>HR &amp; Workforce</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>AI classification &amp; compensation for local gov HR: job specs, salary benchmarking (Harvard-born)</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
-          <t>None found - 5 roles, none sales</t>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -3789,64 +3788,64 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="24" t="inlineStr">
+      <c r="B1" s="23" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="24" t="inlineStr">
+      <c r="C1" s="23" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="24" t="inlineStr">
+      <c r="D1" s="23" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="24" t="inlineStr">
+      <c r="E1" s="23" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="24" t="inlineStr">
+      <c r="F1" s="23" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Kaizen Labs</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C2" s="26" t="n">
+      <c r="C2" s="25" t="n">
         <v>2021</v>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="24" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>Modern resident services platform born in parks &amp; rec registration; $21M Series A (NEA, a16z, Accel)</t>
         </is>
       </c>
-      <c r="F2" s="27" t="inlineStr">
-        <is>
-          <t>Yes - AE, remote+travel</t>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -3874,39 +3873,39 @@
           <t>Parks &amp; rec program management and booking platform founded by early Uber employees</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Ent AE, SF/East Coast</t>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Account Executive (San Francisco, CA)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>RecDesk</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Old Lyme, CT</t>
         </is>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="25" t="n">
         <v>2007</v>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E4" s="25" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Simple recreation management software for small-town rec departments (Clubessential Holdings)</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
-        <is>
-          <t>None found - QA eng only</t>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
         </is>
       </c>
     </row>
@@ -3936,37 +3935,37 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Vermont Systems</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Essex Junction, VT</t>
         </is>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="25" t="n">
         <v>1985</v>
       </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E6" s="25" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>RecTrac - the legacy standard for municipal parks &amp; rec management (Clubessential Holdings)</t>
         </is>
       </c>
-      <c r="F6" s="28" t="inlineStr">
-        <is>
-          <t>None found - site board: no sales</t>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
         </is>
       </c>
     </row>
@@ -3996,37 +3995,37 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Unknown - GlobalPay AE unverified</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Amilia</t>
         </is>
       </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Montreal, QC, Canada</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="25" t="n">
         <v>2009</v>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E8" s="25" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>SmartRec activity registration and facility management platform</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
-        <is>
-          <t>Yes - Ent AE Public Sector US</t>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -4054,39 +4053,39 @@
           <t>Recreation and community center management platform, now part of Xplor</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>None found - Xplor: no rec AEs</t>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Bryan, TX)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Daxko</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Birmingham, AL</t>
         </is>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="25" t="n">
         <v>1998</v>
       </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E10" s="25" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Membership and operations software for YMCAs, JCCs, and community rec centers</t>
         </is>
       </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>None found - own site: 0 open jobs</t>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 429 for https://www.daxko.com/compa</t>
         </is>
       </c>
     </row>
@@ -4116,37 +4115,37 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>None found - AE removed May 26</t>
+          <t>Unknown - HTTP 404 for https://leagueapps.com/care</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>SportsEngine</t>
         </is>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Minneapolis, MN</t>
         </is>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="25" t="n">
         <v>2008</v>
       </c>
-      <c r="D12" s="25" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>Youth Sports &amp; Leagues</t>
         </is>
       </c>
-      <c r="E12" s="25" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>NBC Sports-owned registration, scheduling, and website platform for youth sports</t>
         </is>
       </c>
-      <c r="F12" s="28" t="inlineStr">
-        <is>
-          <t>None found - post expired</t>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://www.sportsengine.co</t>
         </is>
       </c>
     </row>
@@ -4174,39 +4173,39 @@
           <t>Team and league management apps for youth sports, with a business tier for rec orgs</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Enterprise AE, remote</t>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Account Executive (Remote)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>TeamSideline</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Roseville, CA</t>
         </is>
       </c>
-      <c r="C14" s="26" t="n">
+      <c r="C14" s="25" t="n">
         <v>2007</v>
       </c>
-      <c r="D14" s="25" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>Youth Sports &amp; Leagues</t>
         </is>
       </c>
-      <c r="E14" s="25" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>League management, registration, and scheduling for rec departments and leagues</t>
         </is>
       </c>
-      <c r="F14" s="28" t="inlineStr">
-        <is>
-          <t>None found - no open roles</t>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -4241,64 +4240,64 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" s="28" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" s="28" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" s="28" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" s="28" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="29" t="inlineStr">
+      <c r="F1" s="28" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>Raptor Technologies</t>
         </is>
       </c>
-      <c r="B2" s="30" t="inlineStr">
+      <c r="B2" s="29" t="inlineStr">
         <is>
           <t>Houston, TX</t>
         </is>
       </c>
-      <c r="C2" s="31" t="n">
+      <c r="C2" s="30" t="n">
         <v>2002</v>
       </c>
-      <c r="D2" s="30" t="inlineStr">
+      <c r="D2" s="29" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E2" s="30" t="inlineStr">
+      <c r="E2" s="29" t="inlineStr">
         <is>
           <t>Visitor management, emergency management, and reunification software for K-12</t>
         </is>
       </c>
-      <c r="F2" s="32" t="inlineStr">
-        <is>
-          <t>None found - site: 2 jobs, no sales</t>
+      <c r="F2" s="31" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive  (Remote - US)</t>
         </is>
       </c>
     </row>
@@ -4326,39 +4325,39 @@
           <t>CrisisAlert wearable panic buttons for school staff; 18M+ people covered</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Sales Exec, Central</t>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ZeroEyes</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Conshohocken, PA</t>
         </is>
       </c>
-      <c r="C4" s="31" t="n">
+      <c r="C4" s="30" t="n">
         <v>2018</v>
       </c>
-      <c r="D4" s="30" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E4" s="30" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>AI gun detection layered onto existing school security cameras</t>
         </is>
       </c>
       <c r="F4" s="32" t="inlineStr">
         <is>
-          <t>None found - tech/ops only</t>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -4388,37 +4387,37 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>None found - LA AE closed</t>
+          <t>Unknown - HTTP 403 for https://www.evolvtechnology</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Gaggle</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Bloomington, IL</t>
         </is>
       </c>
-      <c r="C6" s="31" t="n">
+      <c r="C6" s="30" t="n">
         <v>1999</v>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E6" s="30" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>Monitors school email/docs for self-harm and threat signals</t>
         </is>
       </c>
       <c r="F6" s="33" t="inlineStr">
         <is>
-          <t>Yes - Regional SM, West</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -4448,37 +4447,37 @@
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>Yes - New Business Exec</t>
+          <t>Sales (non-AE) - Senior Sales Coach only</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Securly</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>San Jose, CA</t>
         </is>
       </c>
-      <c r="C8" s="31" t="n">
+      <c r="C8" s="30" t="n">
         <v>2013</v>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>Cloud web filtering and student safety monitoring</t>
         </is>
       </c>
-      <c r="F8" s="32" t="inlineStr">
-        <is>
-          <t>None found - talent community only</t>
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive, Large/Enterpris (United States of A)</t>
         </is>
       </c>
     </row>
@@ -4508,37 +4507,37 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>None found - BD Mgr closed</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>HopSkipDrive</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Los Angeles, CA</t>
         </is>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="30" t="n">
         <v>2014</v>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>Vetted small-vehicle student rides supplementing district bus fleets</t>
         </is>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Reg Acct Mgrs + SDR</t>
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>Yes - Regional Account Manager (Remote USA )</t>
         </is>
       </c>
     </row>
@@ -4566,39 +4565,39 @@
           <t>School bus telematics, electronic inspections, and ridership tracking</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Yes - 2 Strat Sales Dir remote</t>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Edulog</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Missoula, MT</t>
         </is>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="30" t="n">
         <v>1977</v>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D12" s="29" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="E12" s="30" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>Longtime standard for school bus routing and planning software</t>
         </is>
       </c>
-      <c r="F12" s="32" t="inlineStr">
-        <is>
-          <t>None found - IT tech only</t>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -4626,39 +4625,39 @@
           <t>Student information system giant plus enrollment, comms, and analytics</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Inside Sales AM</t>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Infinite Campus</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>Blaine, MN</t>
         </is>
       </c>
-      <c r="C14" s="31" t="n">
+      <c r="C14" s="30" t="n">
         <v>1993</v>
       </c>
-      <c r="D14" s="30" t="inlineStr">
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>Operations &amp; SIS</t>
         </is>
       </c>
-      <c r="E14" s="30" t="inlineStr">
+      <c r="E14" s="29" t="inlineStr">
         <is>
           <t>SIS serving thousands of districts nationwide</t>
         </is>
       </c>
-      <c r="F14" s="32" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -4686,39 +4685,39 @@
           <t>K-12 HR, absence and substitute management, and operations software</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Strategic AE + RSM</t>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 403 for https://careers.frontlineed</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>ParentSquare</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>Santa Barbara, CA</t>
         </is>
       </c>
-      <c r="C16" s="31" t="n">
+      <c r="C16" s="30" t="n">
         <v>2011</v>
       </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>Operations &amp; SIS</t>
         </is>
       </c>
-      <c r="E16" s="30" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>Unified school-home communication platform</t>
         </is>
       </c>
       <c r="F16" s="32" t="inlineStr">
         <is>
-          <t>None found - CS/RevOps only</t>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -4753,64 +4752,64 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="35" t="inlineStr">
+      <c r="B1" s="34" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="35" t="inlineStr">
+      <c r="C1" s="34" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="35" t="inlineStr">
+      <c r="D1" s="34" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="35" t="inlineStr">
+      <c r="E1" s="34" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="35" t="inlineStr">
+      <c r="F1" s="34" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>Cubic Transportation Systems</t>
         </is>
       </c>
-      <c r="B2" s="36" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
         <is>
           <t>San Diego, CA</t>
         </is>
       </c>
-      <c r="C2" s="37" t="n">
+      <c r="C2" s="36" t="n">
         <v>1951</v>
       </c>
-      <c r="D2" s="36" t="inlineStr">
+      <c r="D2" s="35" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E2" s="36" t="inlineStr">
+      <c r="E2" s="35" t="inlineStr">
         <is>
           <t>Fare collection giant behind OMNY, Opal, and Oyster; ITS systems</t>
         </is>
       </c>
-      <c r="F2" s="38" t="inlineStr">
-        <is>
-          <t>Yes - Sales AE on own Workday</t>
+      <c r="F2" s="37" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager - East Coast (2 Locations)</t>
         </is>
       </c>
     </row>
@@ -4838,39 +4837,39 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>None found - 21 roles, none sales</t>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Via</t>
         </is>
       </c>
-      <c r="B4" s="36" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C4" s="37" t="n">
+      <c r="C4" s="36" t="n">
         <v>2012</v>
       </c>
-      <c r="D4" s="36" t="inlineStr">
+      <c r="D4" s="35" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E4" s="36" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t>On-demand transit, paratransit, and network planning software for agencies</t>
         </is>
       </c>
-      <c r="F4" s="38" t="inlineStr">
-        <is>
-          <t>Yes - Sr Ent AE, Eastern US</t>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive, Western Europe  (Paris)</t>
         </is>
       </c>
     </row>
@@ -4900,37 +4899,37 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>None found - ATS: 0 openings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>Swiftly</t>
         </is>
       </c>
-      <c r="B6" s="36" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="36" t="n">
         <v>2014</v>
       </c>
-      <c r="D6" s="36" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E6" s="36" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>Yes - SMB Sales Mgr</t>
+      <c r="F6" s="37" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Manager — Talent Co (United States)</t>
         </is>
       </c>
     </row>
@@ -4958,39 +4957,39 @@
           <t>Justride fare payments SaaS used by hundreds of agencies</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>None found - site: 7 roles, none sales</t>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Customer Success Manager - UK only</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>Token Transit</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="C8" s="36" t="n">
         <v>2015</v>
       </c>
-      <c r="D8" s="36" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F8" s="39" t="inlineStr">
-        <is>
-          <t>Unknown - site JS-walled</t>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>Unknown - page too small - likely JS-rendered</t>
         </is>
       </c>
     </row>
@@ -5020,37 +5019,37 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Unknown - ADP portal JS-walled</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>ParkMobile</t>
         </is>
       </c>
-      <c r="B10" s="36" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Atlanta, GA</t>
         </is>
       </c>
-      <c r="C10" s="37" t="n">
+      <c r="C10" s="36" t="n">
         <v>2008</v>
       </c>
-      <c r="D10" s="36" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>Parking &amp; Curb</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F10" s="39" t="inlineStr">
-        <is>
-          <t>None found - no sales jobs</t>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
@@ -5080,37 +5079,37 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - careers JS-walled</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Automotus</t>
         </is>
       </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Los Angeles, CA</t>
         </is>
       </c>
-      <c r="C12" s="37" t="n">
+      <c r="C12" s="36" t="n">
         <v>2017</v>
       </c>
-      <c r="D12" s="36" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>Parking &amp; Curb</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
-        <is>
-          <t>None found - marketing only</t>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5139,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - no ATS on file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten page-scan sales detection; discover 6 ATS endpoints; add bamboohr
scan_pagetext used SALES_ORG_NON_AE_PAT, which is tuned for discrete job
titles where every string is already known to be one. On free page text it
matched navigation - 'Customer Success' and 'Channel' are nav sections on half
these marketing sites - so 6 of 10 page-scan 'Sales (non-AE)' verdicts were
reading chrome, not reqs. Page scans now require the role noun too.

ATS discovery over the 24 companies with no board on file found 6 usable
endpoints (3 of them BambooHR, whose public careers/list JSON is now a
supported fetcher). Frontline Wildfire, Routeware, Polco and Euna each turned
out to have an open AE req that was invisible before.

Left Rave (-> Motorola) and RoadBotics (-> Michelin) unwired: their careers
pages redirect to the parent's Workday, and reporting a parent req as the
subsidiary's would be a false Yes.
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -195,7 +195,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -213,8 +212,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -899,7 +898,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -957,9 +956,9 @@
           <t>Exterior retardant/foam systems and app-based wildfire defense for homes and HOAs</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Territory Manager - LA (Los Angeles, CA)</t>
         </is>
       </c>
     </row>
@@ -1557,9 +1556,9 @@
           <t>Real-time EMS-to-hospital communication and patient handoff platform</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -1889,9 +1888,9 @@
           <t>Routing, in-cab fleet tech, and resident apps for waste operations</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive - Municipalities</t>
         </is>
       </c>
     </row>
@@ -2669,9 +2668,9 @@
           <t>Lead service line inventories, sampling, and compliance software</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -3211,9 +3210,9 @@
           <t>Community surveys, benchmarking, and budget simulation (owns National Research Center)</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Madison, WI)</t>
         </is>
       </c>
     </row>
@@ -3421,9 +3420,9 @@
           <t>Procurement, budgeting, and grants suite - Bonfire, Questica, eCivis (formerly GTY)</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Account Executive (Mid-Market)</t>
         </is>
       </c>
     </row>
@@ -3661,9 +3660,9 @@
           <t>Public-sector HR suite: recruiting, onboarding, and performance</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -3691,9 +3690,9 @@
           <t>Workforce management giant (Kronos + Ultimate merger) with large gov base</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -3788,62 +3787,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="23" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Kaizen Labs</t>
         </is>
       </c>
-      <c r="B2" s="24" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C2" s="25" t="n">
+      <c r="C2" s="24" t="n">
         <v>2021</v>
       </c>
-      <c r="D2" s="24" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Modern resident services platform born in parks &amp; rec registration; $21M Series A (NEA, a16z, Accel)</t>
         </is>
       </c>
-      <c r="F2" s="26" t="inlineStr">
+      <c r="F2" s="25" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -3880,30 +3879,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>RecDesk</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>Old Lyme, CT</t>
         </is>
       </c>
-      <c r="C4" s="25" t="n">
+      <c r="C4" s="24" t="n">
         <v>2007</v>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="23" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Simple recreation management software for small-town rec departments (Clubessential Holdings)</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
         </is>
@@ -3940,30 +3939,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Vermont Systems</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Essex Junction, VT</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="24" t="n">
         <v>1985</v>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="23" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>RecTrac - the legacy standard for municipal parks &amp; rec management (Clubessential Holdings)</t>
         </is>
       </c>
-      <c r="F6" s="27" t="inlineStr">
+      <c r="F6" s="26" t="inlineStr">
         <is>
           <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
         </is>
@@ -4000,30 +3999,30 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Amilia</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Montreal, QC, Canada</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="24" t="n">
         <v>2009</v>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>SmartRec activity registration and facility management platform</t>
         </is>
       </c>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="F8" s="25" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -4060,30 +4059,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>Daxko</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Birmingham, AL</t>
         </is>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="24" t="n">
         <v>1998</v>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>Recreation Management</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>Membership and operations software for YMCAs, JCCs, and community rec centers</t>
         </is>
       </c>
-      <c r="F10" s="26" t="inlineStr">
+      <c r="F10" s="25" t="inlineStr">
         <is>
           <t>Unknown - HTTP 429 for https://www.daxko.com/compa</t>
         </is>
@@ -4120,30 +4119,30 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>SportsEngine</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Minneapolis, MN</t>
         </is>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="C12" s="24" t="n">
         <v>2008</v>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>Youth Sports &amp; Leagues</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>NBC Sports-owned registration, scheduling, and website platform for youth sports</t>
         </is>
       </c>
-      <c r="F12" s="26" t="inlineStr">
+      <c r="F12" s="25" t="inlineStr">
         <is>
           <t>Unknown - HTTP 404 for https://www.sportsengine.co</t>
         </is>
@@ -4180,30 +4179,30 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>TeamSideline</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Roseville, CA</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="24" t="n">
         <v>2007</v>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="23" t="inlineStr">
         <is>
           <t>Youth Sports &amp; Leagues</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="23" t="inlineStr">
         <is>
           <t>League management, registration, and scheduling for rec departments and leagues</t>
         </is>
       </c>
-      <c r="F14" s="26" t="inlineStr">
+      <c r="F14" s="25" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
@@ -4240,62 +4239,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="28" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="28" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Raptor Technologies</t>
         </is>
       </c>
-      <c r="B2" s="29" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>Houston, TX</t>
         </is>
       </c>
-      <c r="C2" s="30" t="n">
+      <c r="C2" s="29" t="n">
         <v>2002</v>
       </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E2" s="29" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>Visitor management, emergency management, and reunification software for K-12</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>Yes - Senior Account Executive  (Remote - US)</t>
         </is>
@@ -4332,32 +4331,32 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ZeroEyes</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>Conshohocken, PA</t>
         </is>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="29" t="n">
         <v>2018</v>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>AI gun detection layered onto existing school security cameras</t>
         </is>
       </c>
-      <c r="F4" s="32" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -4392,30 +4391,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Gaggle</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>Bloomington, IL</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="29" t="n">
         <v>1999</v>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>Monitors school email/docs for self-harm and threat signals</t>
         </is>
       </c>
-      <c r="F6" s="33" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -4452,30 +4451,30 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Securly</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>San Jose, CA</t>
         </is>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="29" t="n">
         <v>2013</v>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="28" t="inlineStr">
         <is>
           <t>School Safety</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>Cloud web filtering and student safety monitoring</t>
         </is>
       </c>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Large/Enterpris (United States of A)</t>
         </is>
@@ -4512,30 +4511,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>HopSkipDrive</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Los Angeles, CA</t>
         </is>
       </c>
-      <c r="C10" s="30" t="n">
+      <c r="C10" s="29" t="n">
         <v>2014</v>
       </c>
-      <c r="D10" s="29" t="inlineStr">
+      <c r="D10" s="28" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>Vetted small-vehicle student rides supplementing district bus fleets</t>
         </is>
       </c>
-      <c r="F10" s="31" t="inlineStr">
+      <c r="F10" s="30" t="inlineStr">
         <is>
           <t>Yes - Regional Account Manager (Remote USA )</t>
         </is>
@@ -4572,30 +4571,30 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Edulog</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Missoula, MT</t>
         </is>
       </c>
-      <c r="C12" s="30" t="n">
+      <c r="C12" s="29" t="n">
         <v>1977</v>
       </c>
-      <c r="D12" s="29" t="inlineStr">
+      <c r="D12" s="28" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Longtime standard for school bus routing and planning software</t>
         </is>
       </c>
-      <c r="F12" s="33" t="inlineStr">
+      <c r="F12" s="31" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -4632,30 +4631,30 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Infinite Campus</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>Blaine, MN</t>
         </is>
       </c>
-      <c r="C14" s="30" t="n">
+      <c r="C14" s="29" t="n">
         <v>1993</v>
       </c>
-      <c r="D14" s="29" t="inlineStr">
+      <c r="D14" s="28" t="inlineStr">
         <is>
           <t>Operations &amp; SIS</t>
         </is>
       </c>
-      <c r="E14" s="29" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>SIS serving thousands of districts nationwide</t>
         </is>
       </c>
-      <c r="F14" s="33" t="inlineStr">
+      <c r="F14" s="31" t="inlineStr">
         <is>
           <t>Unknown - page scan found no listings</t>
         </is>
@@ -4692,25 +4691,25 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>ParentSquare</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Santa Barbara, CA</t>
         </is>
       </c>
-      <c r="C16" s="30" t="n">
+      <c r="C16" s="29" t="n">
         <v>2011</v>
       </c>
-      <c r="D16" s="29" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>Operations &amp; SIS</t>
         </is>
       </c>
-      <c r="E16" s="29" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>Unified school-home communication platform</t>
         </is>
@@ -4752,62 +4751,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C1" s="34" t="inlineStr">
+      <c r="C1" s="33" t="inlineStr">
         <is>
           <t>Year Founded</t>
         </is>
       </c>
-      <c r="D1" s="34" t="inlineStr">
+      <c r="D1" s="33" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="34" t="inlineStr">
+      <c r="E1" s="33" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" s="34" t="inlineStr">
+      <c r="F1" s="33" t="inlineStr">
         <is>
           <t>Hiring AEs? (8/16/26)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="34" t="inlineStr">
         <is>
           <t>Cubic Transportation Systems</t>
         </is>
       </c>
-      <c r="B2" s="35" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>San Diego, CA</t>
         </is>
       </c>
-      <c r="C2" s="36" t="n">
+      <c r="C2" s="35" t="n">
         <v>1951</v>
       </c>
-      <c r="D2" s="35" t="inlineStr">
+      <c r="D2" s="34" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E2" s="35" t="inlineStr">
+      <c r="E2" s="34" t="inlineStr">
         <is>
           <t>Fare collection giant behind OMNY, Opal, and Oyster; ITS systems</t>
         </is>
       </c>
-      <c r="F2" s="37" t="inlineStr">
+      <c r="F2" s="36" t="inlineStr">
         <is>
           <t>Yes - Account Manager - East Coast (2 Locations)</t>
         </is>
@@ -4837,37 +4836,37 @@
           <t>Bus ITS: CAD/AVL, real-time passenger info, and fleet health</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>Via</t>
         </is>
       </c>
-      <c r="B4" s="35" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="C4" s="36" t="n">
+      <c r="C4" s="35" t="n">
         <v>2012</v>
       </c>
-      <c r="D4" s="35" t="inlineStr">
+      <c r="D4" s="34" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E4" s="35" t="inlineStr">
+      <c r="E4" s="34" t="inlineStr">
         <is>
           <t>On-demand transit, paratransit, and network planning software for agencies</t>
         </is>
       </c>
-      <c r="F4" s="37" t="inlineStr">
+      <c r="F4" s="36" t="inlineStr">
         <is>
           <t>Yes - Account Executive, Western Europe  (Paris)</t>
         </is>
@@ -4904,30 +4903,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>Swiftly</t>
         </is>
       </c>
-      <c r="B6" s="35" t="inlineStr">
+      <c r="B6" s="34" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="C6" s="35" t="n">
         <v>2014</v>
       </c>
-      <c r="D6" s="35" t="inlineStr">
+      <c r="D6" s="34" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E6" s="35" t="inlineStr">
+      <c r="E6" s="34" t="inlineStr">
         <is>
           <t>Real-time transit data: arrival predictions and on-time performance</t>
         </is>
       </c>
-      <c r="F6" s="37" t="inlineStr">
+      <c r="F6" s="36" t="inlineStr">
         <is>
           <t>Yes - Senior Account Manager — Talent Co (United States)</t>
         </is>
@@ -4964,30 +4963,30 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>Token Transit</t>
         </is>
       </c>
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="34" t="inlineStr">
         <is>
           <t>San Francisco, CA</t>
         </is>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="35" t="n">
         <v>2015</v>
       </c>
-      <c r="D8" s="35" t="inlineStr">
+      <c r="D8" s="34" t="inlineStr">
         <is>
           <t>Transit Tech</t>
         </is>
       </c>
-      <c r="E8" s="35" t="inlineStr">
+      <c r="E8" s="34" t="inlineStr">
         <is>
           <t>Mobile fare payment app covering 200+ North American agencies</t>
         </is>
       </c>
-      <c r="F8" s="38" t="inlineStr">
+      <c r="F8" s="37" t="inlineStr">
         <is>
           <t>Unknown - page too small - likely JS-rendered</t>
         </is>
@@ -5024,30 +5023,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="35" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>ParkMobile</t>
         </is>
       </c>
-      <c r="B10" s="35" t="inlineStr">
+      <c r="B10" s="34" t="inlineStr">
         <is>
           <t>Atlanta, GA</t>
         </is>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="35" t="n">
         <v>2008</v>
       </c>
-      <c r="D10" s="35" t="inlineStr">
+      <c r="D10" s="34" t="inlineStr">
         <is>
           <t>Parking &amp; Curb</t>
         </is>
       </c>
-      <c r="E10" s="35" t="inlineStr">
+      <c r="E10" s="34" t="inlineStr">
         <is>
           <t>Leading mobile parking payments app (EasyPark Group)</t>
         </is>
       </c>
-      <c r="F10" s="38" t="inlineStr">
+      <c r="F10" s="37" t="inlineStr">
         <is>
           <t>Unknown - no ATS on file</t>
         </is>
@@ -5077,37 +5076,37 @@
           <t>Smart single-space parking meters and enforcement systems</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - no ATS on file</t>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Sr. Client Success Manager only</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>Automotus</t>
         </is>
       </c>
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>Los Angeles, CA</t>
         </is>
       </c>
-      <c r="C12" s="36" t="n">
+      <c r="C12" s="35" t="n">
         <v>2017</v>
       </c>
-      <c r="D12" s="35" t="inlineStr">
+      <c r="D12" s="34" t="inlineStr">
         <is>
           <t>Parking &amp; Curb</t>
         </is>
       </c>
-      <c r="E12" s="35" t="inlineStr">
+      <c r="E12" s="34" t="inlineStr">
         <is>
           <t>Computer vision curb management and automated loading-zone payments</t>
         </is>
       </c>
-      <c r="F12" s="38" t="inlineStr">
+      <c r="F12" s="37" t="inlineStr">
         <is>
           <t>None found</t>
         </is>

</xml_diff>

<commit_message>
chore: weekly hiring refresh (2026-08-17)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -718,7 +718,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="F1" s="11" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="F1" s="17" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="F1" s="22" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="F1" s="27" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="F1" s="33" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/16/26)</t>
+          <t>Hiring AEs? (8/17/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Discover 5 ATS endpoints via headless render; stop counting accountants as sales
Rendered the Unknown companies in Chromium and captured the XHR calls their
boards make - a JS-walled board fetches its listings from a JSON endpoint, and
that endpoint is a plain ATS API we can read with requests forever after. So
the browser is a one-off discovery tool, not a CI dependency; the weekly run
stays stdlib-only.

Converted: greyparrot (recruitee), hayden-ai (ashby), urban-sdk (rippling),
leagueapps (greenhouse), zum (lever). Two of those - leagueapps and urban-sdk -
were dead 404 URLs that no amount of page-scanning could have recovered.

Also: SALESY_PAT matched the bare substring 'account', so 'Senior Accountant'
and 'Accounting Manager, Lease & Fixed Assets' were counted as Sales (non-AE).
Finance guard sits after AE_PAT, so 'Account Executive, Accounting Software'
still classifies as an AE req.
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -2008,9 +2008,9 @@
           <t>AI waste-recognition cameras and analytics for sorting plants</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - VP Sales only</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Unknown - no ATS on file</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -2398,9 +2398,9 @@
           <t>Speed, volume, and congestion analytics for public works and police</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>Unknown - HTTP 404 for https://www.urbansdk.com/ca</t>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>Sales (non-AE) -  Customer Support Specialist I, Ac only</t>
+          <t>Sales (non-AE) - Customer Success Manager only</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Bryan, TX)</t>
+          <t>Yes - Account Executive (Amarillo, TX)</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://leagueapps.com/care</t>
+          <t>None found</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>None found</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add iCIMS fetcher; Granicus opens an AE req
iCIMS portals serve a ~600-char shell at the plain URL and put the listing
inside an iframe, which is exactly why these boards looked like JS walls.
?in_iframe=1 returns the real server-rendered list, readable with plain
requests - no browser needed.

Granicus goes Unknown -> Yes on an Enterprise Account Executive (KS/OK/NE),
found in 53 parsed reqs. It had been reported as a confident 'None found'
before the page-scan fix, which is the exact warm door that bug was hiding.

Quarterhill stays Unknown: its careers URL points at a culture page, not its
iCIMS portal, so there is nothing to parse yet.
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -3120,9 +3120,9 @@
           <t>Resident communications (govDelivery), meeting and agenda management, digital services</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Yes - Enterprise Account Executive - KS,</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Yes - Account Executive (Amarillo, TX)</t>
+          <t>Yes - Account Executive (Springfield, IL)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Four new sectors and two General Gov categories for the conference verticals
Courts & Justice, Health & Human Services, Higher Education, and Housing &
Community Dev, each in the house shape (short categories, Suppliers &
Services last, distinct xlsx colors), plus Elections & Voting and Libraries
under General Gov. Empty tabs today, deliberately: the exhibitor sweep's
research pass needs somewhere honest to file a court-tech or Medicaid
vendor, and cramming them into General Gov would muddy the map exactly
where the new coverage is.
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -15,6 +15,10 @@
     <sheet name="Transit &amp; Parking" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Utilities &amp; Energy" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Airports &amp; Aviation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Courts &amp; Justice" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Health &amp; Human Services" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Higher Education" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Housing &amp; Community Dev" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Public Safety'!$A$1:$F$368</definedName>
@@ -25,6 +29,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Transit &amp; Parking'!$A$1:$F$208</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Utilities &amp; Energy'!$A$1:$F$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Airports &amp; Aviation'!$A$1:$F$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Courts &amp; Justice'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Health &amp; Human Services'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Higher Education'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Housing &amp; Community Dev'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -68,7 +76,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -155,6 +163,26 @@
         <fgColor rgb="00F3EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00884EA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00117A65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002471A3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A04000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -182,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -271,6 +299,18 @@
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -348,6 +388,51 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>govtech-dock</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Exported from the govtech-dock repo - edit data/companies.json and re-run scripts/export_xlsx.py rather than editing this file.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>govtech-dock</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Exported from the govtech-dock repo - edit data/companies.json and re-run scripts/export_xlsx.py rather than editing this file.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>govtech-dock</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Exported from the govtech-dock repo - edit data/companies.json and re-run scripts/export_xlsx.py rather than editing this file.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>govtech-dock</author>
@@ -453,6 +538,21 @@
 </file>
 
 <file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>govtech-dock</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Exported from the govtech-dock repo - edit data/companies.json and re-run scripts/export_xlsx.py rather than editing this file.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>govtech-dock</author>
@@ -11214,6 +11314,192 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00117A65"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="55" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C1" s="55" t="inlineStr">
+        <is>
+          <t>Year Founded</t>
+        </is>
+      </c>
+      <c r="D1" s="55" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="55" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="55" t="inlineStr">
+        <is>
+          <t>Hiring AEs? (8/17/26)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Public Health, Benefits &amp; Medicaid Systems, Child &amp; Family Services, Behavioral Health, Aging &amp; Veterans, Workforce &amp; Labor, Suppliers &amp; Services" type="list">
+      <formula1>"Public Health,Benefits &amp; Medicaid Systems,Child &amp; Family Services,Behavioral Health,Aging &amp; Veterans,Workforce &amp; Labor,Suppliers &amp; Services"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002471A3"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="56" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C1" s="56" t="inlineStr">
+        <is>
+          <t>Year Founded</t>
+        </is>
+      </c>
+      <c r="D1" s="56" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="56" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="56" t="inlineStr">
+        <is>
+          <t>Hiring AEs? (8/17/26)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: IT &amp; Administration, Business &amp; Finance, Campus Safety, Suppliers &amp; Services" type="list">
+      <formula1>"IT &amp; Administration,Business &amp; Finance,Campus Safety,Suppliers &amp; Services"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00A04000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="57" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C1" s="57" t="inlineStr">
+        <is>
+          <t>Year Founded</t>
+        </is>
+      </c>
+      <c r="D1" s="57" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="57" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="57" t="inlineStr">
+        <is>
+          <t>Hiring AEs? (8/17/26)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Housing &amp; Assistance, Planning &amp; Economic Development, Suppliers &amp; Services" type="list">
+      <formula1>"Housing &amp; Assistance,Planning &amp; Economic Development,Suppliers &amp; Services"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -30625,8 +30911,8 @@
   </sheetData>
   <autoFilter ref="A1:F450"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Citizen Services, Permitting &amp; Licensing, Finance &amp; ERP, Procurement &amp; Payments, HR &amp; Workforce, Cemetery Management, IT &amp; AI Platforms, Strategy &amp; Performance, Health &amp; Human Services, Elections, Courts &amp; Justice, Suppliers &amp; Services" type="list">
-      <formula1>"Citizen Services,Permitting &amp; Licensing,Finance &amp; ERP,Procurement &amp; Payments,HR &amp; Workforce,Cemetery Management,IT &amp; AI Platforms,Strategy &amp; Performance,Health &amp; Human Services,Elections,Courts &amp; Justice,Suppliers &amp; Services"</formula1>
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Citizen Services, Permitting &amp; Licensing, Finance &amp; ERP, Procurement &amp; Payments, HR &amp; Workforce, Cemetery Management, IT &amp; AI Platforms, Strategy &amp; Performance, Health &amp; Human Services, Elections, Courts &amp; Justice, Elections &amp; Voting, Libraries, Suppliers &amp; Services" type="list">
+      <formula1>"Citizen Services,Permitting &amp; Licensing,Finance &amp; ERP,Procurement &amp; Payments,HR &amp; Workforce,Cemetery Management,IT &amp; AI Platforms,Strategy &amp; Performance,Health &amp; Human Services,Elections,Courts &amp; Justice,Elections &amp; Voting,Libraries,Suppliers &amp; Services"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -51122,4 +51408,66 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00884EA0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C1" s="54" t="inlineStr">
+        <is>
+          <t>Year Founded</t>
+        </is>
+      </c>
+      <c r="D1" s="54" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="54" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="54" t="inlineStr">
+        <is>
+          <t>Hiring AEs? (8/17/26)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick one of: Courts &amp; Case Management, Prosecution &amp; Defense, Probation &amp; Supervision, Suppliers &amp; Services" type="list">
+      <formula1>"Courts &amp; Case Management,Prosecution &amp; Defense,Probation &amp; Supervision,Suppliers &amp; Services"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-08-30)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>None found -  [rendered]</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -6228,7 +6228,7 @@
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
-          <t>None found -  [rendered]</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -11536,7 +11536,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -12854,7 +12854,7 @@
       </c>
       <c r="F48" s="62" t="inlineStr">
         <is>
-          <t>None found -  [rendered]</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -14448,7 +14448,7 @@
       </c>
       <c r="F106" s="62" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="F18" s="68" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 500 for https://recruiting.paylocit</t>
         </is>
       </c>
     </row>
@@ -17488,7 +17488,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -17730,7 +17730,7 @@
       </c>
       <c r="F10" s="74" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.affordablehousi</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -17956,7 +17956,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -25396,7 +25396,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -29008,9 +29008,9 @@
           <t>Connect fund accounting, utility billing, and payments for small and mid-size cities - exhibited at GFOA 2026</t>
         </is>
       </c>
-      <c r="F124" s="21" t="inlineStr">
-        <is>
-          <t>Unknown - page too small - likely JS-rendered</t>
+      <c r="F124" s="23" t="inlineStr">
+        <is>
+          <t>Yes - Account Manager - Sales [rendered]</t>
         </is>
       </c>
     </row>
@@ -30764,9 +30764,9 @@
           <t>Online surplus auction marketplace for 7,500+ governments and schools</t>
         </is>
       </c>
-      <c r="F183" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F183" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 404 for https://municibid.com/caree</t>
         </is>
       </c>
     </row>
@@ -37916,9 +37916,9 @@
           <t>Document, creative and digital experience software - exhibited at NACo 2026, NASCIO 2026, NCSEA 2026, CoSN 2026, APHSA 2026, EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F430" s="22" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Account Manager, Channel Sales only [rendered]</t>
+      <c r="F430" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -39516,7 +39516,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -44152,7 +44152,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -45042,9 +45042,9 @@
           <t>InformaCast mass notification and paging for school districts</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -48398,7 +48398,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -54438,7 +54438,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -57998,7 +57998,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>
@@ -59694,7 +59694,7 @@
       </c>
       <c r="F58" s="51" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.elenium.com/car</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -59904,7 +59904,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 403 for https://www.grab.careers/en</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -61642,7 +61642,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/29/26)</t>
+          <t>Hiring AEs? (8/30/26)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-01)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -2046,9 +2046,9 @@
           <t>License plate readers, gunshot detection, and drone-as-first-responder (Aerodome)</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>Yes - Community Safety Account Executive (Boston, MA)</t>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Associate General Counsel, Revenue only</t>
         </is>
       </c>
     </row>
@@ -8794,7 +8794,7 @@
       </c>
       <c r="F265" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -8854,7 +8854,7 @@
       </c>
       <c r="F267" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -10746,9 +10746,9 @@
           <t>DigiTICKET electronic citation software - exhibited at IACP 2026</t>
         </is>
       </c>
-      <c r="F341" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F341" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11222,7 +11222,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -11724,7 +11724,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="F24" s="62" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 522 for https://www.sandata.com/car</t>
         </is>
       </c>
     </row>
@@ -11904,7 +11904,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 522 for https://www.hhaexchange.com</t>
         </is>
       </c>
     </row>
@@ -14104,9 +14104,9 @@
           <t>EHR and case management software for PACE programs, State Units on Aging, Area Agencies on Aging and community-based aging services organizations - exhibited at USAging 2026</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Sales Director, PACE (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -14214,7 +14214,7 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 522 for https://www.pairin.com/abou</t>
         </is>
       </c>
     </row>
@@ -14482,7 +14482,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -17088,7 +17088,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -17556,7 +17556,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -17674,9 +17674,9 @@
           <t>AI robotic sorting systems for recycling facilities (MRFs)</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Director, Commercial Origination &amp; only [rendered]</t>
         </is>
       </c>
     </row>
@@ -18622,7 +18622,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 525 for https://www.newwaytrucks.co</t>
         </is>
       </c>
     </row>
@@ -22120,7 +22120,7 @@
       </c>
       <c r="F154" s="15" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 522 for https://www.2ndnaturewater.</t>
         </is>
       </c>
     </row>
@@ -22960,7 +22960,7 @@
       </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.cityreportersof</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -23410,7 +23410,7 @@
       </c>
       <c r="F198" s="15" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -24932,7 +24932,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://www.partage.club/ca</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -26388,7 +26388,7 @@
       </c>
       <c r="F58" s="21" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 504 for https://www.amlegal.com/car</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -33592,9 +33592,9 @@
           <t>Strategic plan and KPI reporting (balanced scorecard) for local governments and enterprises</t>
         </is>
       </c>
-      <c r="F303" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F303" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -34030,7 +34030,7 @@
       </c>
       <c r="F318" s="21" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -36352,7 +36352,7 @@
       </c>
       <c r="F399" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -37268,9 +37268,9 @@
           <t>Purchasing card audit and compliance monitoring - exhibited at NIGP 2026</t>
         </is>
       </c>
-      <c r="F432" s="23" t="inlineStr">
-        <is>
-          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
+      <c r="F432" s="21" t="inlineStr">
+        <is>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -38538,7 +38538,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -43048,7 +43048,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -44712,7 +44712,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: Exceeded 30 redirects.</t>
         </is>
       </c>
     </row>
@@ -47174,7 +47174,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -47768,9 +47768,9 @@
           <t>Account-based fare collection and validators for public transit operators</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Yes - Senior Enterprise Account Executiv</t>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Unknown - HTTP 500 for https://ridango.bamboohr.co</t>
         </is>
       </c>
     </row>
@@ -53112,7 +53112,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -56136,7 +56136,7 @@
       </c>
       <c r="F102" s="45" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -56282,7 +56282,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - HTTP 404 for https://ikegps.com/open-pos</t>
         </is>
       </c>
     </row>
@@ -56642,7 +56642,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -56906,7 +56906,7 @@
       </c>
       <c r="F10" s="51" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - network error: HTTPSConnectionPool(host=</t>
         </is>
       </c>
     </row>
@@ -60166,7 +60166,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (8/31/26)</t>
+          <t>Hiring AEs? (9/1/26)</t>
         </is>
       </c>
     </row>
@@ -60682,7 +60682,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Yes - Senior Enterprise Account Executiv (Oakland, Californi)</t>
+          <t>Yes - Senior Enterprise Account Executiv (New York, New York)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: spreadsheet rebuild (2026-09-05)
</commit_message>
<xml_diff>
--- a/exports/GovTech_Company_Tracker.xlsx
+++ b/exports/GovTech_Company_Tracker.xlsx
@@ -942,7 +942,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>Yes - AIoT Sales Director</t>
+          <t>Yes - Sales Director</t>
         </is>
       </c>
     </row>
@@ -7246,7 +7246,7 @@
       </c>
       <c r="F213" s="7" t="inlineStr">
         <is>
-          <t>None found</t>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="F215" s="10" t="inlineStr">
         <is>
-          <t>Yes - Sr Account Executive</t>
+          <t>Yes - Senior Account Manager</t>
         </is>
       </c>
     </row>
@@ -9062,7 +9062,7 @@
       </c>
       <c r="F274" s="4" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 503 for https://norix.com/about-us/</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="F1" s="59" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -14442,7 +14442,7 @@
       </c>
       <c r="F1" s="65" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -15106,9 +15106,9 @@
           <t>Academic scheduling, course demand analytics, and room and event management software for colleges and universities - exhibited at EDUCAUSE 2026</t>
         </is>
       </c>
-      <c r="F24" s="70" t="inlineStr">
-        <is>
-          <t>Yes - Account Executive (Expansion) (Overland Park, KS,)</t>
+      <c r="F24" s="69" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - Senior Client Success Lead only</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="F1" s="71" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="F10" s="74" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.affordablehousi</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="F1" s="12" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -17666,7 +17666,7 @@
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Climate Tech ( (West - Remote)</t>
+          <t>Yes - Account Executive - Climate Tech ( (Remote East Coast )</t>
         </is>
       </c>
     </row>
@@ -18872,7 +18872,7 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>Yes - Strategic Account Executive (North Carolina_Rem)</t>
+          <t>Yes - Strategic Account Executive (Tennessee_Remote_C)</t>
         </is>
       </c>
     </row>
@@ -21084,7 +21084,7 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>Yes - Account Executive - Government (Remote)</t>
+          <t>Yes - Account Executive - Government (Ca (Remote)</t>
         </is>
       </c>
     </row>
@@ -23064,7 +23064,7 @@
       </c>
       <c r="F188" s="16" t="inlineStr">
         <is>
-          <t>Yes - Account Executive, Enterprise - Mo (United States - Re)</t>
+          <t>Yes - Account Executive, Enterprise - Ce (United States - Re)</t>
         </is>
       </c>
     </row>
@@ -24646,7 +24646,7 @@
       </c>
       <c r="F1" s="18" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -29774,7 +29774,7 @@
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
-          <t>Unknown - HTTP 404 for https://lcptracker.com/care</t>
+          <t>Unknown - HTTP 500 for https://lcptracker.com/care</t>
         </is>
       </c>
     </row>
@@ -30164,7 +30164,7 @@
       </c>
       <c r="F188" s="22" t="inlineStr">
         <is>
-          <t>Sales (non-AE) - Deployment Operations &amp; Customer S only</t>
+          <t>Sales (non-AE) - Founding GTM Engineer only</t>
         </is>
       </c>
     </row>
@@ -33644,9 +33644,9 @@
           <t>Strategic planning, performance measurement, and public dashboards built for local government</t>
         </is>
       </c>
-      <c r="F307" s="9" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - Remote Account Payable Specialist only</t>
+      <c r="F307" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Senior Account Executive - Public  (Canada)</t>
         </is>
       </c>
     </row>
@@ -38524,7 +38524,7 @@
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -40132,7 +40132,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.swimtopia.com/c</t>
         </is>
       </c>
     </row>
@@ -43034,7 +43034,7 @@
       </c>
       <c r="F1" s="30" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -45714,9 +45714,9 @@
           <t>School and district websites, apps and communications for public schools</t>
         </is>
       </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>None found</t>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>Yes - Sales Executive (Remote Worker - N/)</t>
         </is>
       </c>
     </row>
@@ -47130,7 +47130,7 @@
       </c>
       <c r="F1" s="36" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -53002,7 +53002,7 @@
       </c>
       <c r="F1" s="42" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -54500,9 +54500,9 @@
           <t>Grid software, ADMS and transmission equipment for public and investor utilities</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>Yes - AE-type role (page scan) [page scan - verify]</t>
         </is>
       </c>
     </row>
@@ -55724,9 +55724,9 @@
           <t>SaaS deployment, project, and asset lifecycle management for infrastructure programs; sold to agencies via Carahsoft (SEWP V, NASPO)</t>
         </is>
       </c>
-      <c r="F92" s="47" t="inlineStr">
-        <is>
-          <t>Sales (non-AE) - sales roles, none AE</t>
+      <c r="F92" s="45" t="inlineStr">
+        <is>
+          <t>Unknown - page scan found no listings</t>
         </is>
       </c>
     </row>
@@ -56532,7 +56532,7 @@
       </c>
       <c r="F1" s="48" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>
@@ -58016,9 +58016,9 @@
           <t>Baggage handling systems and terminal logistics for airports</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Unknown - page scan found no listings</t>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Sales (non-AE) - sales roles, none AE</t>
         </is>
       </c>
     </row>
@@ -58378,7 +58378,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Unknown - page scan found no listings</t>
+          <t>Unknown - HTTP 403 for https://www.grab.careers/en</t>
         </is>
       </c>
     </row>
@@ -60056,7 +60056,7 @@
       </c>
       <c r="F1" s="54" t="inlineStr">
         <is>
-          <t>Hiring AEs? (9/4/26)</t>
+          <t>Hiring AEs? (9/5/26)</t>
         </is>
       </c>
     </row>

</xml_diff>